<commit_message>
Update Excel data analyst practice file
</commit_message>
<xml_diff>
--- a/ExcelForDA.xlsx
+++ b/ExcelForDA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data-Analyst-Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD252CCE-0446-4B40-A7C8-300D1E65399C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96874B97-BD8B-4D28-950B-FC74A4899366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{9812301C-C18C-46F2-AD5A-E6FD016C11F9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{9812301C-C18C-46F2-AD5A-E6FD016C11F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Entry And Basic Formatting" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Sorting " sheetId="4" r:id="rId4"/>
     <sheet name="Filter" sheetId="5" r:id="rId5"/>
     <sheet name="Table Creation" sheetId="6" r:id="rId6"/>
+    <sheet name="Logical formula" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Filter!$A$2:$J$52</definedName>
@@ -32,8 +34,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId7"/>
-        <x14:slicerCache r:id="rId8"/>
+        <x14:slicerCache r:id="rId9"/>
+        <x14:slicerCache r:id="rId10"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -52,8 +54,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1861" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2174" uniqueCount="93">
   <si>
     <t>OrderID</t>
   </si>
@@ -347,6 +371,12 @@
   </si>
   <si>
     <t>Total Sal</t>
+  </si>
+  <si>
+    <t>Sales Grade</t>
+  </si>
+  <si>
+    <t>Bonus</t>
   </si>
 </sst>
 </file>
@@ -696,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -750,21 +780,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -801,20 +816,75 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="19">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -833,44 +903,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="9" tint="0.79998168889431442"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color auto="1"/>
-        </left>
-        <right style="medium">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1069,13 +1101,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thick">
           <color auto="1"/>
         </left>
@@ -1091,28 +1116,49 @@
       </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
+      <border outline="0">
+        <bottom style="medium">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="9" tint="0.79998168889431442"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color auto="1"/>
+        </left>
+        <right style="medium">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1147,8 +1193,8 @@
       <xdr:row>28</xdr:row>
       <xdr:rowOff>144781</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="2" name="Category">
@@ -1171,7 +1217,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -1225,8 +1271,8 @@
       <xdr:row>14</xdr:row>
       <xdr:rowOff>137161</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="PaymentMode">
@@ -1249,7 +1295,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -1321,7 +1367,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0A40A2E6-9EF9-4A23-B4F1-36607D28E91E}" name="Table2" displayName="Table2" ref="A2:K52" totalsRowShown="0" headerRowDxfId="1" dataDxfId="2" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0A40A2E6-9EF9-4A23-B4F1-36607D28E91E}" name="Table2" displayName="Table2" ref="A2:K52" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15" totalsRowBorderDxfId="14">
   <autoFilter ref="A2:K52" xr:uid="{0A40A2E6-9EF9-4A23-B4F1-36607D28E91E}">
     <filterColumn colId="5">
       <filters>
@@ -1336,17 +1382,17 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{F20047A1-28CA-4A2E-9700-EE85CD967777}" name="OrderID" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{38D9ABC4-7A81-4317-8CAA-E808FA6A19E6}" name="Date" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{83CF5A52-5AA1-420E-A0EB-5A173A27E6F4}" name="Customer" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{9137BB94-ADC5-4CE6-89AE-AA2D1B9D0E25}" name="City" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{1433C48A-095C-457E-99CD-EDEEE68C5541}" name="Product" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{DD554F32-43E4-46AC-976E-F414A48908A6}" name="Category" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{5A226ED8-2D5A-49C5-BBF9-B33FBC37A3AD}" name="Quantity" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{2B6B6351-50CA-4CE2-A6DF-A1CB48D6DA61}" name="UnitPrice" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{2FD782BE-192E-4C3F-9D63-33A3852C92BA}" name="PaymentMode" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{C89072BA-5DCB-44F9-A7AE-F51D0432AA7C}" name="Salesperson" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{79D75163-9AC6-4E8C-B655-F7AAF75FA590}" name="Total Sal" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F20047A1-28CA-4A2E-9700-EE85CD967777}" name="OrderID" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{38D9ABC4-7A81-4317-8CAA-E808FA6A19E6}" name="Date" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{83CF5A52-5AA1-420E-A0EB-5A173A27E6F4}" name="Customer" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{9137BB94-ADC5-4CE6-89AE-AA2D1B9D0E25}" name="City" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{1433C48A-095C-457E-99CD-EDEEE68C5541}" name="Product" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{DD554F32-43E4-46AC-976E-F414A48908A6}" name="Category" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{5A226ED8-2D5A-49C5-BBF9-B33FBC37A3AD}" name="Quantity" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{2B6B6351-50CA-4CE2-A6DF-A1CB48D6DA61}" name="UnitPrice" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{2FD782BE-192E-4C3F-9D63-33A3852C92BA}" name="PaymentMode" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{C89072BA-5DCB-44F9-A7AE-F51D0432AA7C}" name="Salesperson" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{79D75163-9AC6-4E8C-B655-F7AAF75FA590}" name="Total Sal" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="1"/>
 </table>
@@ -6843,12 +6889,12 @@
     <row r="52" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="D2:D51">
-    <cfRule type="containsText" dxfId="18" priority="7" operator="containsText" text="Lucknow">
+    <cfRule type="containsText" dxfId="2" priority="7" operator="containsText" text="Lucknow">
       <formula>NOT(ISERROR(SEARCH("Lucknow",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F51">
-    <cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="Accessories">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Accessories">
       <formula>NOT(ISERROR(SEARCH("Accessories",F2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6867,7 +6913,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I51">
-    <cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="UPI">
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="UPI">
       <formula>NOT(ISERROR(SEARCH("UPI",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6921,90 +6967,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="3" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27"/>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="A1" s="40"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
     </row>
     <row r="2" spans="1:21" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
     </row>
     <row r="3" spans="1:21" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="27"/>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
     </row>
     <row r="4" spans="1:21" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
     </row>
     <row r="5" spans="1:21" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="40"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="L6" s="25" t="s">
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="L6" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="26"/>
-      <c r="T6" s="26"/>
-      <c r="U6" s="26"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="42"/>
+      <c r="O6" s="42"/>
+      <c r="P6" s="42"/>
+      <c r="Q6" s="42"/>
+      <c r="R6" s="42"/>
+      <c r="S6" s="42"/>
+      <c r="T6" s="42"/>
+      <c r="U6" s="42"/>
     </row>
     <row r="7" spans="1:21" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
@@ -8000,18 +8046,18 @@
     </row>
     <row r="23" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
     </row>
     <row r="26" spans="1:21" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="4" t="s">
@@ -8608,18 +8654,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="43" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
     </row>
     <row r="2" spans="1:10" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
@@ -10288,57 +10334,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="44"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="37"/>
     </row>
     <row r="2" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="36" t="s">
+      <c r="F2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="36" t="s">
+      <c r="G2" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="36" t="s">
+      <c r="I2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="38" t="s">
+      <c r="J2" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="36" t="s">
+      <c r="K2" s="31" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="33">
+      <c r="A3" s="28">
         <v>1001</v>
       </c>
       <c r="B3" s="6">
@@ -10365,16 +10411,16 @@
       <c r="I3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="34" t="s">
+      <c r="J3" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="41">
+      <c r="K3" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>110000</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="33">
+      <c r="A4" s="28">
         <v>1002</v>
       </c>
       <c r="B4" s="6">
@@ -10401,16 +10447,16 @@
       <c r="I4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="34" t="s">
+      <c r="J4" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="41">
+      <c r="K4" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>66000</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="33">
+      <c r="A5" s="28">
         <v>1003</v>
       </c>
       <c r="B5" s="6">
@@ -10437,13 +10483,13 @@
       <c r="I5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="34" t="s">
+      <c r="J5" s="29" t="s">
         <v>26</v>
       </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="33">
+      <c r="A6" s="28">
         <v>1004</v>
       </c>
       <c r="B6" s="6">
@@ -10470,13 +10516,13 @@
       <c r="I6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="34" t="s">
+      <c r="J6" s="29" t="s">
         <v>15</v>
       </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="33">
+      <c r="A7" s="28">
         <v>1005</v>
       </c>
       <c r="B7" s="6">
@@ -10503,13 +10549,13 @@
       <c r="I7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="34" t="s">
+      <c r="J7" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="33">
+      <c r="A8" s="28">
         <v>1006</v>
       </c>
       <c r="B8" s="6">
@@ -10536,16 +10582,16 @@
       <c r="I8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="J8" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="K8" s="41">
+      <c r="K8" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>30000</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="33">
+      <c r="A9" s="28">
         <v>1007</v>
       </c>
       <c r="B9" s="6">
@@ -10572,16 +10618,16 @@
       <c r="I9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="J9" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K9" s="41">
+      <c r="K9" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>62000</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="33">
+      <c r="A10" s="28">
         <v>1008</v>
       </c>
       <c r="B10" s="6">
@@ -10608,13 +10654,13 @@
       <c r="I10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J10" s="34" t="s">
+      <c r="J10" s="29" t="s">
         <v>15</v>
       </c>
       <c r="K10" s="3"/>
     </row>
     <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="33">
+      <c r="A11" s="28">
         <v>1009</v>
       </c>
       <c r="B11" s="6">
@@ -10641,16 +10687,16 @@
       <c r="I11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="34" t="s">
+      <c r="J11" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="41">
+      <c r="K11" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>36000</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="33">
+      <c r="A12" s="28">
         <v>1010</v>
       </c>
       <c r="B12" s="6">
@@ -10677,13 +10723,13 @@
       <c r="I12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="34" t="s">
+      <c r="J12" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K12" s="3"/>
     </row>
     <row r="13" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="33">
+      <c r="A13" s="28">
         <v>1011</v>
       </c>
       <c r="B13" s="6">
@@ -10710,13 +10756,13 @@
       <c r="I13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="34" t="s">
+      <c r="J13" s="29" t="s">
         <v>26</v>
       </c>
       <c r="K13" s="3"/>
     </row>
     <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="33">
+      <c r="A14" s="28">
         <v>1012</v>
       </c>
       <c r="B14" s="6">
@@ -10743,16 +10789,16 @@
       <c r="I14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="34" t="s">
+      <c r="J14" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K14" s="41">
+      <c r="K14" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>58000</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="33">
+      <c r="A15" s="28">
         <v>1013</v>
       </c>
       <c r="B15" s="6">
@@ -10779,16 +10825,16 @@
       <c r="I15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K15" s="41">
+      <c r="K15" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>40500</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="33">
+      <c r="A16" s="28">
         <v>1014</v>
       </c>
       <c r="B16" s="6">
@@ -10815,13 +10861,13 @@
       <c r="I16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K16" s="3"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="33">
+      <c r="A17" s="28">
         <v>1015</v>
       </c>
       <c r="B17" s="6">
@@ -10848,16 +10894,16 @@
       <c r="I17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="34" t="s">
+      <c r="J17" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="41">
+      <c r="K17" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>11000</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="33">
+      <c r="A18" s="28">
         <v>1016</v>
       </c>
       <c r="B18" s="6">
@@ -10884,16 +10930,16 @@
       <c r="I18" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J18" s="34" t="s">
+      <c r="J18" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K18" s="41">
+      <c r="K18" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>75000</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="33">
+      <c r="A19" s="28">
         <v>1017</v>
       </c>
       <c r="B19" s="6">
@@ -10920,13 +10966,13 @@
       <c r="I19" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J19" s="34" t="s">
+      <c r="J19" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K19" s="3"/>
     </row>
     <row r="20" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="33">
+      <c r="A20" s="28">
         <v>1018</v>
       </c>
       <c r="B20" s="6">
@@ -10953,13 +10999,13 @@
       <c r="I20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J20" s="34" t="s">
+      <c r="J20" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="33">
+      <c r="A21" s="28">
         <v>1019</v>
       </c>
       <c r="B21" s="6">
@@ -10986,16 +11032,16 @@
       <c r="I21" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J21" s="34" t="s">
+      <c r="J21" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="41">
+      <c r="K21" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>120000</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="33">
+      <c r="A22" s="28">
         <v>1020</v>
       </c>
       <c r="B22" s="6">
@@ -11022,16 +11068,16 @@
       <c r="I22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J22" s="34" t="s">
+      <c r="J22" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K22" s="41">
+      <c r="K22" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>16000</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="33">
+      <c r="A23" s="28">
         <v>1021</v>
       </c>
       <c r="B23" s="6">
@@ -11058,16 +11104,16 @@
       <c r="I23" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J23" s="34" t="s">
+      <c r="J23" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K23" s="41">
+      <c r="K23" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>18000</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="33">
+      <c r="A24" s="28">
         <v>1022</v>
       </c>
       <c r="B24" s="6">
@@ -11094,13 +11140,13 @@
       <c r="I24" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="34" t="s">
+      <c r="J24" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K24" s="3"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="33">
+      <c r="A25" s="28">
         <v>1023</v>
       </c>
       <c r="B25" s="6">
@@ -11127,16 +11173,16 @@
       <c r="I25" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J25" s="34" t="s">
+      <c r="J25" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K25" s="41">
+      <c r="K25" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>42000</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="33">
+      <c r="A26" s="28">
         <v>1024</v>
       </c>
       <c r="B26" s="6">
@@ -11163,13 +11209,13 @@
       <c r="I26" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J26" s="34" t="s">
+      <c r="J26" s="29" t="s">
         <v>15</v>
       </c>
       <c r="K26" s="3"/>
     </row>
     <row r="27" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="33">
+      <c r="A27" s="28">
         <v>1025</v>
       </c>
       <c r="B27" s="6">
@@ -11196,13 +11242,13 @@
       <c r="I27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J27" s="34" t="s">
+      <c r="J27" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K27" s="3"/>
     </row>
     <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="33">
+      <c r="A28" s="28">
         <v>1026</v>
       </c>
       <c r="B28" s="6">
@@ -11229,16 +11275,16 @@
       <c r="I28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J28" s="34" t="s">
+      <c r="J28" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="K28" s="41">
+      <c r="K28" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>65000</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="33">
+      <c r="A29" s="28">
         <v>1027</v>
       </c>
       <c r="B29" s="6">
@@ -11265,16 +11311,16 @@
       <c r="I29" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J29" s="34" t="s">
+      <c r="J29" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K29" s="41">
+      <c r="K29" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>29000</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="33">
+      <c r="A30" s="28">
         <v>1028</v>
       </c>
       <c r="B30" s="6">
@@ -11301,16 +11347,16 @@
       <c r="I30" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J30" s="34" t="s">
+      <c r="J30" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K30" s="41">
+      <c r="K30" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>25500</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="33">
+      <c r="A31" s="28">
         <v>1029</v>
       </c>
       <c r="B31" s="6">
@@ -11337,13 +11383,13 @@
       <c r="I31" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J31" s="34" t="s">
+      <c r="J31" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K31" s="3"/>
     </row>
     <row r="32" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="33">
+      <c r="A32" s="28">
         <v>1030</v>
       </c>
       <c r="B32" s="6">
@@ -11370,13 +11416,13 @@
       <c r="I32" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="34" t="s">
+      <c r="J32" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K32" s="3"/>
     </row>
     <row r="33" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="33">
+      <c r="A33" s="28">
         <v>1031</v>
       </c>
       <c r="B33" s="6">
@@ -11403,13 +11449,13 @@
       <c r="I33" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J33" s="34" t="s">
+      <c r="J33" s="29" t="s">
         <v>26</v>
       </c>
       <c r="K33" s="3"/>
     </row>
     <row r="34" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="33">
+      <c r="A34" s="28">
         <v>1032</v>
       </c>
       <c r="B34" s="6">
@@ -11436,13 +11482,13 @@
       <c r="I34" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J34" s="34" t="s">
+      <c r="J34" s="29" t="s">
         <v>15</v>
       </c>
       <c r="K34" s="3"/>
     </row>
     <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="33">
+      <c r="A35" s="28">
         <v>1033</v>
       </c>
       <c r="B35" s="6">
@@ -11469,16 +11515,16 @@
       <c r="I35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J35" s="34" t="s">
+      <c r="J35" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K35" s="41">
+      <c r="K35" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>114000</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="33">
+      <c r="A36" s="28">
         <v>1034</v>
       </c>
       <c r="B36" s="6">
@@ -11505,13 +11551,13 @@
       <c r="I36" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J36" s="34" t="s">
+      <c r="J36" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K36" s="3"/>
     </row>
     <row r="37" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="33">
+      <c r="A37" s="28">
         <v>1035</v>
       </c>
       <c r="B37" s="6">
@@ -11538,16 +11584,16 @@
       <c r="I37" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J37" s="34" t="s">
+      <c r="J37" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K37" s="41">
+      <c r="K37" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>20000</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="33">
+      <c r="A38" s="28">
         <v>1036</v>
       </c>
       <c r="B38" s="6">
@@ -11574,16 +11620,16 @@
       <c r="I38" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J38" s="34" t="s">
+      <c r="J38" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K38" s="41">
+      <c r="K38" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>78000</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="33">
+      <c r="A39" s="28">
         <v>1037</v>
       </c>
       <c r="B39" s="6">
@@ -11610,13 +11656,13 @@
       <c r="I39" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J39" s="34" t="s">
+      <c r="J39" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K39" s="3"/>
     </row>
     <row r="40" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="33">
+      <c r="A40" s="28">
         <v>1038</v>
       </c>
       <c r="B40" s="6">
@@ -11643,13 +11689,13 @@
       <c r="I40" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J40" s="34" t="s">
+      <c r="J40" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K40" s="3"/>
     </row>
     <row r="41" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="33">
+      <c r="A41" s="28">
         <v>1039</v>
       </c>
       <c r="B41" s="6">
@@ -11676,16 +11722,16 @@
       <c r="I41" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J41" s="34" t="s">
+      <c r="J41" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K41" s="41">
+      <c r="K41" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>61000</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="33">
+      <c r="A42" s="28">
         <v>1040</v>
       </c>
       <c r="B42" s="6">
@@ -11712,16 +11758,16 @@
       <c r="I42" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J42" s="34" t="s">
+      <c r="J42" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K42" s="41">
+      <c r="K42" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>25000</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="33">
+      <c r="A43" s="28">
         <v>1041</v>
       </c>
       <c r="B43" s="6">
@@ -11748,16 +11794,16 @@
       <c r="I43" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J43" s="34" t="s">
+      <c r="J43" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K43" s="41">
+      <c r="K43" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>9500</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="33">
+      <c r="A44" s="28">
         <v>1042</v>
       </c>
       <c r="B44" s="6">
@@ -11784,13 +11830,13 @@
       <c r="I44" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J44" s="34" t="s">
+      <c r="J44" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K44" s="3"/>
     </row>
     <row r="45" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="33">
+      <c r="A45" s="28">
         <v>1043</v>
       </c>
       <c r="B45" s="6">
@@ -11817,16 +11863,16 @@
       <c r="I45" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J45" s="34" t="s">
+      <c r="J45" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K45" s="41">
+      <c r="K45" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>52000</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="33">
+      <c r="A46" s="28">
         <v>1044</v>
       </c>
       <c r="B46" s="6">
@@ -11853,13 +11899,13 @@
       <c r="I46" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J46" s="34" t="s">
+      <c r="J46" s="29" t="s">
         <v>15</v>
       </c>
       <c r="K46" s="3"/>
     </row>
     <row r="47" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="33">
+      <c r="A47" s="28">
         <v>1045</v>
       </c>
       <c r="B47" s="6">
@@ -11886,13 +11932,13 @@
       <c r="I47" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J47" s="34" t="s">
+      <c r="J47" s="29" t="s">
         <v>16</v>
       </c>
       <c r="K47" s="3"/>
     </row>
     <row r="48" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="33">
+      <c r="A48" s="28">
         <v>1046</v>
       </c>
       <c r="B48" s="6">
@@ -11919,13 +11965,13 @@
       <c r="I48" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J48" s="34" t="s">
+      <c r="J48" s="29" t="s">
         <v>20</v>
       </c>
       <c r="K48" s="3"/>
     </row>
     <row r="49" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="33">
+      <c r="A49" s="28">
         <v>1047</v>
       </c>
       <c r="B49" s="6">
@@ -11952,16 +11998,16 @@
       <c r="I49" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J49" s="34" t="s">
+      <c r="J49" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="K49" s="41">
+      <c r="K49" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>42000</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="33">
+      <c r="A50" s="28">
         <v>1048</v>
       </c>
       <c r="B50" s="6">
@@ -11988,16 +12034,16 @@
       <c r="I50" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J50" s="34" t="s">
+      <c r="J50" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="K50" s="41">
+      <c r="K50" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>18400</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="33">
+      <c r="A51" s="28">
         <v>1049</v>
       </c>
       <c r="B51" s="6">
@@ -12024,46 +12070,46 @@
       <c r="I51" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J51" s="34" t="s">
+      <c r="J51" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="K51" s="41">
+      <c r="K51" s="36">
         <f>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[UnitPrice]]</f>
         <v>60000</v>
       </c>
     </row>
     <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="39">
+      <c r="A52" s="34">
         <v>1050</v>
       </c>
-      <c r="B52" s="30">
+      <c r="B52" s="25">
         <v>46259</v>
       </c>
-      <c r="C52" s="31" t="s">
+      <c r="C52" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="D52" s="31" t="s">
+      <c r="D52" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="E52" s="31" t="s">
+      <c r="E52" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="F52" s="31" t="s">
+      <c r="F52" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="G52" s="31">
+      <c r="G52" s="26">
         <v>4</v>
       </c>
-      <c r="H52" s="32">
+      <c r="H52" s="27">
         <v>2700</v>
       </c>
-      <c r="I52" s="31" t="s">
+      <c r="I52" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="J52" s="40" t="s">
+      <c r="J52" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="K52" s="31"/>
+      <c r="K52" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -12082,4 +12128,2078 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57CBF72A-0E93-45FF-9270-C5E3252F3AA5}">
+  <dimension ref="A1:M51"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="45" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" s="45" t="s">
+        <v>91</v>
+      </c>
+      <c r="M1" s="45" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="47">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="48">
+        <v>46235</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="47">
+        <v>2</v>
+      </c>
+      <c r="H2" s="49">
+        <v>55000</v>
+      </c>
+      <c r="I2" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" s="50">
+        <f>G2*H2</f>
+        <v>110000</v>
+      </c>
+      <c r="L2" t="str" cm="1">
+        <f t="array" ref="L2">_xlfn.IFS(K2&gt;=100000,"Great Sale",K2&gt;=50000,"Good Sale",K2&gt;=30,"Avg Sale",K2&lt;=10000,"Poor Sale")</f>
+        <v>Great Sale</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="47">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="48">
+        <v>46235</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="47">
+        <v>3</v>
+      </c>
+      <c r="H3" s="49">
+        <v>22000</v>
+      </c>
+      <c r="I3" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="50">
+        <f t="shared" ref="K3:K51" si="0">G3*H3</f>
+        <v>66000</v>
+      </c>
+      <c r="L3" t="str" cm="1">
+        <f t="array" ref="L3">_xlfn.IFS(K3&gt;=100000,"Great Sale",K3&gt;=50000,"Good Sale",K3&gt;=30,"Avg Sale",K3&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="47">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="48">
+        <v>46236</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="47">
+        <v>5</v>
+      </c>
+      <c r="H4" s="49">
+        <v>1200</v>
+      </c>
+      <c r="I4" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="50">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+      <c r="L4" t="str" cm="1">
+        <f t="array" ref="L4">_xlfn.IFS(K4&gt;=100000,"Great Sale",K4&gt;=50000,"Good Sale",K4&gt;=30,"Avg Sale",K4&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="47">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="48">
+        <v>46236</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="47">
+        <v>4</v>
+      </c>
+      <c r="H5" s="49">
+        <v>800</v>
+      </c>
+      <c r="I5" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" s="50">
+        <f t="shared" si="0"/>
+        <v>3200</v>
+      </c>
+      <c r="L5" t="str" cm="1">
+        <f t="array" ref="L5">_xlfn.IFS(K5&gt;=100000,"Great Sale",K5&gt;=50000,"Good Sale",K5&gt;=30,"Avg Sale",K5&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="47">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="48">
+        <v>46237</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="47">
+        <v>2</v>
+      </c>
+      <c r="H6" s="49">
+        <v>2500</v>
+      </c>
+      <c r="I6" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="50">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+      <c r="L6" t="str" cm="1">
+        <f t="array" ref="L6">_xlfn.IFS(K6&gt;=100000,"Great Sale",K6&gt;=50000,"Good Sale",K6&gt;=30,"Avg Sale",K6&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="47">
+        <v>1006</v>
+      </c>
+      <c r="B7" s="48">
+        <v>46237</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="47">
+        <v>2</v>
+      </c>
+      <c r="H7" s="49">
+        <v>15000</v>
+      </c>
+      <c r="I7" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="50">
+        <f t="shared" si="0"/>
+        <v>30000</v>
+      </c>
+      <c r="L7" t="str" cm="1">
+        <f t="array" ref="L7">_xlfn.IFS(K7&gt;=100000,"Great Sale",K7&gt;=50000,"Good Sale",K7&gt;=30,"Avg Sale",K7&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="47">
+        <v>1007</v>
+      </c>
+      <c r="B8" s="48">
+        <v>46238</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="47">
+        <v>1</v>
+      </c>
+      <c r="H8" s="49">
+        <v>62000</v>
+      </c>
+      <c r="I8" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="50">
+        <f t="shared" si="0"/>
+        <v>62000</v>
+      </c>
+      <c r="L8" t="str" cm="1">
+        <f t="array" ref="L8">_xlfn.IFS(K8&gt;=100000,"Great Sale",K8&gt;=50000,"Good Sale",K8&gt;=30,"Avg Sale",K8&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" s="47">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="48">
+        <v>46238</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="47">
+        <v>2</v>
+      </c>
+      <c r="H9" s="49">
+        <v>9500</v>
+      </c>
+      <c r="I9" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" s="50">
+        <f t="shared" si="0"/>
+        <v>19000</v>
+      </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" ref="L9">_xlfn.IFS(K9&gt;=100000,"Great Sale",K9&gt;=50000,"Good Sale",K9&gt;=30,"Avg Sale",K9&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="47">
+        <v>1009</v>
+      </c>
+      <c r="B10" s="48">
+        <v>46239</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="47" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="47">
+        <v>2</v>
+      </c>
+      <c r="H10" s="49">
+        <v>18000</v>
+      </c>
+      <c r="I10" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="50">
+        <f t="shared" si="0"/>
+        <v>36000</v>
+      </c>
+      <c r="L10" t="str" cm="1">
+        <f t="array" ref="L10">_xlfn.IFS(K10&gt;=100000,"Great Sale",K10&gt;=50000,"Good Sale",K10&gt;=30,"Avg Sale",K10&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="47">
+        <v>1010</v>
+      </c>
+      <c r="B11" s="48">
+        <v>46239</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="47">
+        <v>3</v>
+      </c>
+      <c r="H11" s="49">
+        <v>1500</v>
+      </c>
+      <c r="I11" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="50">
+        <f t="shared" si="0"/>
+        <v>4500</v>
+      </c>
+      <c r="L11" t="str" cm="1">
+        <f t="array" ref="L11">_xlfn.IFS(K11&gt;=100000,"Great Sale",K11&gt;=50000,"Good Sale",K11&gt;=30,"Avg Sale",K11&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="47">
+        <v>1011</v>
+      </c>
+      <c r="B12" s="48">
+        <v>46240</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="47">
+        <v>6</v>
+      </c>
+      <c r="H12" s="49">
+        <v>700</v>
+      </c>
+      <c r="I12" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="50">
+        <f t="shared" si="0"/>
+        <v>4200</v>
+      </c>
+      <c r="L12" t="str" cm="1">
+        <f t="array" ref="L12">_xlfn.IFS(K12&gt;=100000,"Great Sale",K12&gt;=50000,"Good Sale",K12&gt;=30,"Avg Sale",K12&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="47">
+        <v>1012</v>
+      </c>
+      <c r="B13" s="48">
+        <v>46240</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="47">
+        <v>1</v>
+      </c>
+      <c r="H13" s="49">
+        <v>58000</v>
+      </c>
+      <c r="I13" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K13" s="50">
+        <f t="shared" si="0"/>
+        <v>58000</v>
+      </c>
+      <c r="L13" t="str" cm="1">
+        <f t="array" ref="L13">_xlfn.IFS(K13&gt;=100000,"Great Sale",K13&gt;=50000,"Good Sale",K13&gt;=30,"Avg Sale",K13&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="47">
+        <v>1013</v>
+      </c>
+      <c r="B14" s="48">
+        <v>46241</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="47">
+        <v>3</v>
+      </c>
+      <c r="H14" s="49">
+        <v>13500</v>
+      </c>
+      <c r="I14" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="50">
+        <f t="shared" si="0"/>
+        <v>40500</v>
+      </c>
+      <c r="L14" t="str" cm="1">
+        <f t="array" ref="L14">_xlfn.IFS(K14&gt;=100000,"Great Sale",K14&gt;=50000,"Good Sale",K14&gt;=30,"Avg Sale",K14&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="47">
+        <v>1014</v>
+      </c>
+      <c r="B15" s="48">
+        <v>46241</v>
+      </c>
+      <c r="C15" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="47">
+        <v>4</v>
+      </c>
+      <c r="H15" s="49">
+        <v>2200</v>
+      </c>
+      <c r="I15" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="50">
+        <f t="shared" si="0"/>
+        <v>8800</v>
+      </c>
+      <c r="L15" t="str" cm="1">
+        <f t="array" ref="L15">_xlfn.IFS(K15&gt;=100000,"Great Sale",K15&gt;=50000,"Good Sale",K15&gt;=30,"Avg Sale",K15&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="47">
+        <v>1015</v>
+      </c>
+      <c r="B16" s="48">
+        <v>46242</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="47">
+        <v>1</v>
+      </c>
+      <c r="H16" s="49">
+        <v>11000</v>
+      </c>
+      <c r="I16" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="50">
+        <f t="shared" si="0"/>
+        <v>11000</v>
+      </c>
+      <c r="L16" t="str" cm="1">
+        <f t="array" ref="L16">_xlfn.IFS(K16&gt;=100000,"Great Sale",K16&gt;=50000,"Good Sale",K16&gt;=30,"Avg Sale",K16&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="47">
+        <v>1016</v>
+      </c>
+      <c r="B17" s="48">
+        <v>46242</v>
+      </c>
+      <c r="C17" s="47" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="47">
+        <v>3</v>
+      </c>
+      <c r="H17" s="49">
+        <v>25000</v>
+      </c>
+      <c r="I17" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" s="50">
+        <f t="shared" si="0"/>
+        <v>75000</v>
+      </c>
+      <c r="L17" t="str" cm="1">
+        <f t="array" ref="L17">_xlfn.IFS(K17&gt;=100000,"Great Sale",K17&gt;=50000,"Good Sale",K17&gt;=30,"Avg Sale",K17&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" s="47">
+        <v>1017</v>
+      </c>
+      <c r="B18" s="48">
+        <v>46243</v>
+      </c>
+      <c r="C18" s="47" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="47">
+        <v>5</v>
+      </c>
+      <c r="H18" s="49">
+        <v>1300</v>
+      </c>
+      <c r="I18" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K18" s="50">
+        <f t="shared" si="0"/>
+        <v>6500</v>
+      </c>
+      <c r="L18" t="str" cm="1">
+        <f t="array" ref="L18">_xlfn.IFS(K18&gt;=100000,"Great Sale",K18&gt;=50000,"Good Sale",K18&gt;=30,"Avg Sale",K18&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="47">
+        <v>1018</v>
+      </c>
+      <c r="B19" s="48">
+        <v>46243</v>
+      </c>
+      <c r="C19" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" s="47">
+        <v>8</v>
+      </c>
+      <c r="H19" s="49">
+        <v>650</v>
+      </c>
+      <c r="I19" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K19" s="50">
+        <f t="shared" si="0"/>
+        <v>5200</v>
+      </c>
+      <c r="L19" t="str" cm="1">
+        <f t="array" ref="L19">_xlfn.IFS(K19&gt;=100000,"Great Sale",K19&gt;=50000,"Good Sale",K19&gt;=30,"Avg Sale",K19&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="47">
+        <v>1019</v>
+      </c>
+      <c r="B20" s="48">
+        <v>46244</v>
+      </c>
+      <c r="C20" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="47">
+        <v>2</v>
+      </c>
+      <c r="H20" s="49">
+        <v>60000</v>
+      </c>
+      <c r="I20" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K20" s="50">
+        <f t="shared" si="0"/>
+        <v>120000</v>
+      </c>
+      <c r="L20" t="str" cm="1">
+        <f t="array" ref="L20">_xlfn.IFS(K20&gt;=100000,"Great Sale",K20&gt;=50000,"Good Sale",K20&gt;=30,"Avg Sale",K20&lt;=10000,"Poor Sale")</f>
+        <v>Great Sale</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="47">
+        <v>1020</v>
+      </c>
+      <c r="B21" s="48">
+        <v>46244</v>
+      </c>
+      <c r="C21" s="47" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="47">
+        <v>1</v>
+      </c>
+      <c r="H21" s="49">
+        <v>16000</v>
+      </c>
+      <c r="I21" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" s="50">
+        <f t="shared" si="0"/>
+        <v>16000</v>
+      </c>
+      <c r="L21" t="str" cm="1">
+        <f t="array" ref="L21">_xlfn.IFS(K21&gt;=100000,"Great Sale",K21&gt;=50000,"Good Sale",K21&gt;=30,"Avg Sale",K21&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="47">
+        <v>1021</v>
+      </c>
+      <c r="B22" s="48">
+        <v>46245</v>
+      </c>
+      <c r="C22" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="47">
+        <v>2</v>
+      </c>
+      <c r="H22" s="49">
+        <v>9000</v>
+      </c>
+      <c r="I22" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J22" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K22" s="50">
+        <f t="shared" si="0"/>
+        <v>18000</v>
+      </c>
+      <c r="L22" t="str" cm="1">
+        <f t="array" ref="L22">_xlfn.IFS(K22&gt;=100000,"Great Sale",K22&gt;=50000,"Good Sale",K22&gt;=30,"Avg Sale",K22&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="47">
+        <v>1022</v>
+      </c>
+      <c r="B23" s="48">
+        <v>46245</v>
+      </c>
+      <c r="C23" s="47" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F23" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="47">
+        <v>3</v>
+      </c>
+      <c r="H23" s="49">
+        <v>2800</v>
+      </c>
+      <c r="I23" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J23" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K23" s="50">
+        <f t="shared" si="0"/>
+        <v>8400</v>
+      </c>
+      <c r="L23" t="str" cm="1">
+        <f t="array" ref="L23">_xlfn.IFS(K23&gt;=100000,"Great Sale",K23&gt;=50000,"Good Sale",K23&gt;=30,"Avg Sale",K23&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="47">
+        <v>1023</v>
+      </c>
+      <c r="B24" s="48">
+        <v>46246</v>
+      </c>
+      <c r="C24" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="47">
+        <v>2</v>
+      </c>
+      <c r="H24" s="49">
+        <v>21000</v>
+      </c>
+      <c r="I24" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J24" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K24" s="50">
+        <f t="shared" si="0"/>
+        <v>42000</v>
+      </c>
+      <c r="L24" t="str" cm="1">
+        <f t="array" ref="L24">_xlfn.IFS(K24&gt;=100000,"Great Sale",K24&gt;=50000,"Good Sale",K24&gt;=30,"Avg Sale",K24&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="47">
+        <v>1024</v>
+      </c>
+      <c r="B25" s="48">
+        <v>46246</v>
+      </c>
+      <c r="C25" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G25" s="47">
+        <v>4</v>
+      </c>
+      <c r="H25" s="49">
+        <v>1400</v>
+      </c>
+      <c r="I25" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" s="50">
+        <f t="shared" si="0"/>
+        <v>5600</v>
+      </c>
+      <c r="L25" t="str" cm="1">
+        <f t="array" ref="L25">_xlfn.IFS(K25&gt;=100000,"Great Sale",K25&gt;=50000,"Good Sale",K25&gt;=30,"Avg Sale",K25&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="47">
+        <v>1025</v>
+      </c>
+      <c r="B26" s="48">
+        <v>46247</v>
+      </c>
+      <c r="C26" s="47" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E26" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G26" s="47">
+        <v>5</v>
+      </c>
+      <c r="H26" s="49">
+        <v>750</v>
+      </c>
+      <c r="I26" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J26" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K26" s="50">
+        <f t="shared" si="0"/>
+        <v>3750</v>
+      </c>
+      <c r="L26" t="str" cm="1">
+        <f t="array" ref="L26">_xlfn.IFS(K26&gt;=100000,"Great Sale",K26&gt;=50000,"Good Sale",K26&gt;=30,"Avg Sale",K26&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="47">
+        <v>1026</v>
+      </c>
+      <c r="B27" s="48">
+        <v>46247</v>
+      </c>
+      <c r="C27" s="47" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="47">
+        <v>1</v>
+      </c>
+      <c r="H27" s="49">
+        <v>65000</v>
+      </c>
+      <c r="I27" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K27" s="50">
+        <f t="shared" si="0"/>
+        <v>65000</v>
+      </c>
+      <c r="L27" t="str" cm="1">
+        <f t="array" ref="L27">_xlfn.IFS(K27&gt;=100000,"Great Sale",K27&gt;=50000,"Good Sale",K27&gt;=30,"Avg Sale",K27&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="47">
+        <v>1027</v>
+      </c>
+      <c r="B28" s="48">
+        <v>46248</v>
+      </c>
+      <c r="C28" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="47">
+        <v>2</v>
+      </c>
+      <c r="H28" s="49">
+        <v>14500</v>
+      </c>
+      <c r="I28" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K28" s="50">
+        <f t="shared" si="0"/>
+        <v>29000</v>
+      </c>
+      <c r="L28" t="str" cm="1">
+        <f t="array" ref="L28">_xlfn.IFS(K28&gt;=100000,"Great Sale",K28&gt;=50000,"Good Sale",K28&gt;=30,"Avg Sale",K28&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="47">
+        <v>1028</v>
+      </c>
+      <c r="B29" s="48">
+        <v>46248</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="47">
+        <v>3</v>
+      </c>
+      <c r="H29" s="49">
+        <v>8500</v>
+      </c>
+      <c r="I29" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J29" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K29" s="50">
+        <f t="shared" si="0"/>
+        <v>25500</v>
+      </c>
+      <c r="L29" t="str" cm="1">
+        <f t="array" ref="L29">_xlfn.IFS(K29&gt;=100000,"Great Sale",K29&gt;=50000,"Good Sale",K29&gt;=30,"Avg Sale",K29&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" s="47">
+        <v>1029</v>
+      </c>
+      <c r="B30" s="48">
+        <v>46249</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="47">
+        <v>1</v>
+      </c>
+      <c r="H30" s="49">
+        <v>23000</v>
+      </c>
+      <c r="I30" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J30" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K30" s="50">
+        <f t="shared" si="0"/>
+        <v>23000</v>
+      </c>
+      <c r="L30" t="str" cm="1">
+        <f t="array" ref="L30">_xlfn.IFS(K30&gt;=100000,"Great Sale",K30&gt;=50000,"Good Sale",K30&gt;=30,"Avg Sale",K30&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="47">
+        <v>1030</v>
+      </c>
+      <c r="B31" s="48">
+        <v>46249</v>
+      </c>
+      <c r="C31" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E31" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F31" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G31" s="47">
+        <v>2</v>
+      </c>
+      <c r="H31" s="49">
+        <v>3000</v>
+      </c>
+      <c r="I31" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J31" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K31" s="50">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+      <c r="L31" t="str" cm="1">
+        <f t="array" ref="L31">_xlfn.IFS(K31&gt;=100000,"Great Sale",K31&gt;=50000,"Good Sale",K31&gt;=30,"Avg Sale",K31&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A32" s="47">
+        <v>1031</v>
+      </c>
+      <c r="B32" s="48">
+        <v>46250</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G32" s="47">
+        <v>7</v>
+      </c>
+      <c r="H32" s="49">
+        <v>1100</v>
+      </c>
+      <c r="I32" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J32" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K32" s="50">
+        <f t="shared" si="0"/>
+        <v>7700</v>
+      </c>
+      <c r="L32" t="str" cm="1">
+        <f t="array" ref="L32">_xlfn.IFS(K32&gt;=100000,"Great Sale",K32&gt;=50000,"Good Sale",K32&gt;=30,"Avg Sale",K32&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" s="47">
+        <v>1032</v>
+      </c>
+      <c r="B33" s="48">
+        <v>46250</v>
+      </c>
+      <c r="C33" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G33" s="47">
+        <v>4</v>
+      </c>
+      <c r="H33" s="49">
+        <v>900</v>
+      </c>
+      <c r="I33" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J33" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K33" s="50">
+        <f t="shared" si="0"/>
+        <v>3600</v>
+      </c>
+      <c r="L33" t="str" cm="1">
+        <f t="array" ref="L33">_xlfn.IFS(K33&gt;=100000,"Great Sale",K33&gt;=50000,"Good Sale",K33&gt;=30,"Avg Sale",K33&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34" s="47">
+        <v>1033</v>
+      </c>
+      <c r="B34" s="48">
+        <v>46251</v>
+      </c>
+      <c r="C34" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="47">
+        <v>2</v>
+      </c>
+      <c r="H34" s="49">
+        <v>57000</v>
+      </c>
+      <c r="I34" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J34" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K34" s="50">
+        <f t="shared" si="0"/>
+        <v>114000</v>
+      </c>
+      <c r="L34" t="str" cm="1">
+        <f t="array" ref="L34">_xlfn.IFS(K34&gt;=100000,"Great Sale",K34&gt;=50000,"Good Sale",K34&gt;=30,"Avg Sale",K34&lt;=10000,"Poor Sale")</f>
+        <v>Great Sale</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="47">
+        <v>1034</v>
+      </c>
+      <c r="B35" s="48">
+        <v>46251</v>
+      </c>
+      <c r="C35" s="47" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="47">
+        <v>1</v>
+      </c>
+      <c r="H35" s="49">
+        <v>15500</v>
+      </c>
+      <c r="I35" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J35" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K35" s="50">
+        <f t="shared" si="0"/>
+        <v>15500</v>
+      </c>
+      <c r="L35" t="str" cm="1">
+        <f t="array" ref="L35">_xlfn.IFS(K35&gt;=100000,"Great Sale",K35&gt;=50000,"Good Sale",K35&gt;=30,"Avg Sale",K35&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36" s="47">
+        <v>1035</v>
+      </c>
+      <c r="B36" s="48">
+        <v>46252</v>
+      </c>
+      <c r="C36" s="47" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E36" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F36" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="47">
+        <v>2</v>
+      </c>
+      <c r="H36" s="49">
+        <v>10000</v>
+      </c>
+      <c r="I36" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K36" s="50">
+        <f t="shared" si="0"/>
+        <v>20000</v>
+      </c>
+      <c r="L36" t="str" cm="1">
+        <f t="array" ref="L36">_xlfn.IFS(K36&gt;=100000,"Great Sale",K36&gt;=50000,"Good Sale",K36&gt;=30,"Avg Sale",K36&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A37" s="47">
+        <v>1036</v>
+      </c>
+      <c r="B37" s="48">
+        <v>46252</v>
+      </c>
+      <c r="C37" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="D37" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="47">
+        <v>4</v>
+      </c>
+      <c r="H37" s="49">
+        <v>19500</v>
+      </c>
+      <c r="I37" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J37" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K37" s="50">
+        <f t="shared" si="0"/>
+        <v>78000</v>
+      </c>
+      <c r="L37" t="str" cm="1">
+        <f t="array" ref="L37">_xlfn.IFS(K37&gt;=100000,"Great Sale",K37&gt;=50000,"Good Sale",K37&gt;=30,"Avg Sale",K37&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38" s="47">
+        <v>1037</v>
+      </c>
+      <c r="B38" s="48">
+        <v>46253</v>
+      </c>
+      <c r="C38" s="47" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G38" s="47">
+        <v>3</v>
+      </c>
+      <c r="H38" s="49">
+        <v>1600</v>
+      </c>
+      <c r="I38" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J38" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K38" s="50">
+        <f t="shared" si="0"/>
+        <v>4800</v>
+      </c>
+      <c r="L38" t="str" cm="1">
+        <f t="array" ref="L38">_xlfn.IFS(K38&gt;=100000,"Great Sale",K38&gt;=50000,"Good Sale",K38&gt;=30,"Avg Sale",K38&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39" s="47">
+        <v>1038</v>
+      </c>
+      <c r="B39" s="48">
+        <v>46253</v>
+      </c>
+      <c r="C39" s="47" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F39" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G39" s="47">
+        <v>6</v>
+      </c>
+      <c r="H39" s="49">
+        <v>850</v>
+      </c>
+      <c r="I39" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J39" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K39" s="50">
+        <f t="shared" si="0"/>
+        <v>5100</v>
+      </c>
+      <c r="L39" t="str" cm="1">
+        <f t="array" ref="L39">_xlfn.IFS(K39&gt;=100000,"Great Sale",K39&gt;=50000,"Good Sale",K39&gt;=30,"Avg Sale",K39&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" s="47">
+        <v>1039</v>
+      </c>
+      <c r="B40" s="48">
+        <v>46254</v>
+      </c>
+      <c r="C40" s="47" t="s">
+        <v>67</v>
+      </c>
+      <c r="D40" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="47">
+        <v>1</v>
+      </c>
+      <c r="H40" s="49">
+        <v>61000</v>
+      </c>
+      <c r="I40" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J40" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K40" s="50">
+        <f t="shared" si="0"/>
+        <v>61000</v>
+      </c>
+      <c r="L40" t="str" cm="1">
+        <f t="array" ref="L40">_xlfn.IFS(K40&gt;=100000,"Great Sale",K40&gt;=50000,"Good Sale",K40&gt;=30,"Avg Sale",K40&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="47">
+        <v>1040</v>
+      </c>
+      <c r="B41" s="48">
+        <v>46254</v>
+      </c>
+      <c r="C41" s="47" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E41" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="47">
+        <v>2</v>
+      </c>
+      <c r="H41" s="49">
+        <v>12500</v>
+      </c>
+      <c r="I41" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J41" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K41" s="50">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="L41" t="str" cm="1">
+        <f t="array" ref="L41">_xlfn.IFS(K41&gt;=100000,"Great Sale",K41&gt;=50000,"Good Sale",K41&gt;=30,"Avg Sale",K41&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42" s="47">
+        <v>1041</v>
+      </c>
+      <c r="B42" s="48">
+        <v>46255</v>
+      </c>
+      <c r="C42" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D42" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="47">
+        <v>1</v>
+      </c>
+      <c r="H42" s="49">
+        <v>9500</v>
+      </c>
+      <c r="I42" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J42" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K42" s="50">
+        <f t="shared" si="0"/>
+        <v>9500</v>
+      </c>
+      <c r="L42" t="str" cm="1">
+        <f t="array" ref="L42">_xlfn.IFS(K42&gt;=100000,"Great Sale",K42&gt;=50000,"Good Sale",K42&gt;=30,"Avg Sale",K42&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" s="47">
+        <v>1042</v>
+      </c>
+      <c r="B43" s="48">
+        <v>46255</v>
+      </c>
+      <c r="C43" s="47" t="s">
+        <v>69</v>
+      </c>
+      <c r="D43" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F43" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G43" s="47">
+        <v>5</v>
+      </c>
+      <c r="H43" s="49">
+        <v>2400</v>
+      </c>
+      <c r="I43" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J43" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K43" s="50">
+        <f t="shared" si="0"/>
+        <v>12000</v>
+      </c>
+      <c r="L43" t="str" cm="1">
+        <f t="array" ref="L43">_xlfn.IFS(K43&gt;=100000,"Great Sale",K43&gt;=50000,"Good Sale",K43&gt;=30,"Avg Sale",K43&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44" s="47">
+        <v>1043</v>
+      </c>
+      <c r="B44" s="48">
+        <v>46256</v>
+      </c>
+      <c r="C44" s="47" t="s">
+        <v>70</v>
+      </c>
+      <c r="D44" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E44" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" s="47">
+        <v>2</v>
+      </c>
+      <c r="H44" s="49">
+        <v>26000</v>
+      </c>
+      <c r="I44" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J44" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K44" s="50">
+        <f t="shared" si="0"/>
+        <v>52000</v>
+      </c>
+      <c r="L44" t="str" cm="1">
+        <f t="array" ref="L44">_xlfn.IFS(K44&gt;=100000,"Great Sale",K44&gt;=50000,"Good Sale",K44&gt;=30,"Avg Sale",K44&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A45" s="47">
+        <v>1044</v>
+      </c>
+      <c r="B45" s="48">
+        <v>46256</v>
+      </c>
+      <c r="C45" s="47" t="s">
+        <v>71</v>
+      </c>
+      <c r="D45" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F45" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G45" s="47">
+        <v>4</v>
+      </c>
+      <c r="H45" s="49">
+        <v>1250</v>
+      </c>
+      <c r="I45" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J45" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K45" s="50">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+      <c r="L45" t="str" cm="1">
+        <f t="array" ref="L45">_xlfn.IFS(K45&gt;=100000,"Great Sale",K45&gt;=50000,"Good Sale",K45&gt;=30,"Avg Sale",K45&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A46" s="47">
+        <v>1045</v>
+      </c>
+      <c r="B46" s="48">
+        <v>46257</v>
+      </c>
+      <c r="C46" s="47" t="s">
+        <v>72</v>
+      </c>
+      <c r="D46" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E46" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="F46" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G46" s="47">
+        <v>3</v>
+      </c>
+      <c r="H46" s="49">
+        <v>950</v>
+      </c>
+      <c r="I46" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J46" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K46" s="50">
+        <f t="shared" si="0"/>
+        <v>2850</v>
+      </c>
+      <c r="L46" t="str" cm="1">
+        <f t="array" ref="L46">_xlfn.IFS(K46&gt;=100000,"Great Sale",K46&gt;=50000,"Good Sale",K46&gt;=30,"Avg Sale",K46&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47" s="47">
+        <v>1046</v>
+      </c>
+      <c r="B47" s="48">
+        <v>46257</v>
+      </c>
+      <c r="C47" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D47" s="47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="47">
+        <v>2</v>
+      </c>
+      <c r="H47" s="49">
+        <v>59000</v>
+      </c>
+      <c r="I47" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J47" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K47" s="50">
+        <f t="shared" si="0"/>
+        <v>118000</v>
+      </c>
+      <c r="L47" t="str" cm="1">
+        <f t="array" ref="L47">_xlfn.IFS(K47&gt;=100000,"Great Sale",K47&gt;=50000,"Good Sale",K47&gt;=30,"Avg Sale",K47&lt;=10000,"Poor Sale")</f>
+        <v>Great Sale</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48" s="47">
+        <v>1047</v>
+      </c>
+      <c r="B48" s="48">
+        <v>46258</v>
+      </c>
+      <c r="C48" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="D48" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" s="47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" s="47">
+        <v>3</v>
+      </c>
+      <c r="H48" s="49">
+        <v>14000</v>
+      </c>
+      <c r="I48" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J48" s="47" t="s">
+        <v>26</v>
+      </c>
+      <c r="K48" s="50">
+        <f t="shared" si="0"/>
+        <v>42000</v>
+      </c>
+      <c r="L48" t="str" cm="1">
+        <f t="array" ref="L48">_xlfn.IFS(K48&gt;=100000,"Great Sale",K48&gt;=50000,"Good Sale",K48&gt;=30,"Avg Sale",K48&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49" s="47">
+        <v>1048</v>
+      </c>
+      <c r="B49" s="48">
+        <v>46258</v>
+      </c>
+      <c r="C49" s="47" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E49" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="F49" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="47">
+        <v>2</v>
+      </c>
+      <c r="H49" s="49">
+        <v>9200</v>
+      </c>
+      <c r="I49" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="J49" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K49" s="50">
+        <f t="shared" si="0"/>
+        <v>18400</v>
+      </c>
+      <c r="L49" t="str" cm="1">
+        <f t="array" ref="L49">_xlfn.IFS(K49&gt;=100000,"Great Sale",K49&gt;=50000,"Good Sale",K49&gt;=30,"Avg Sale",K49&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" s="47">
+        <v>1049</v>
+      </c>
+      <c r="B50" s="48">
+        <v>46259</v>
+      </c>
+      <c r="C50" s="47" t="s">
+        <v>76</v>
+      </c>
+      <c r="D50" s="47" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="47">
+        <v>3</v>
+      </c>
+      <c r="H50" s="49">
+        <v>20000</v>
+      </c>
+      <c r="I50" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="J50" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="K50" s="50">
+        <f t="shared" si="0"/>
+        <v>60000</v>
+      </c>
+      <c r="L50" t="str" cm="1">
+        <f t="array" ref="L50">_xlfn.IFS(K50&gt;=100000,"Great Sale",K50&gt;=50000,"Good Sale",K50&gt;=30,"Avg Sale",K50&lt;=10000,"Poor Sale")</f>
+        <v>Good Sale</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" s="47">
+        <v>1050</v>
+      </c>
+      <c r="B51" s="48">
+        <v>46259</v>
+      </c>
+      <c r="C51" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="D51" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="E51" s="47" t="s">
+        <v>31</v>
+      </c>
+      <c r="F51" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="G51" s="47">
+        <v>4</v>
+      </c>
+      <c r="H51" s="49">
+        <v>2700</v>
+      </c>
+      <c r="I51" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="J51" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="K51" s="50">
+        <f t="shared" si="0"/>
+        <v>10800</v>
+      </c>
+      <c r="L51" t="str" cm="1">
+        <f t="array" ref="L51">_xlfn.IFS(K51&gt;=100000,"Great Sale",K51&gt;=50000,"Good Sale",K51&gt;=30,"Avg Sale",K51&lt;=10000,"Poor Sale")</f>
+        <v>Avg Sale</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3638228B-6F59-42E2-8B9F-A6E0BC93BE29}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>